<commit_message>
Bumped a lot of working stuff.
</commit_message>
<xml_diff>
--- a/Simulation_studies/cir_parameter_comparison_Xdim2.xlsx
+++ b/Simulation_studies/cir_parameter_comparison_Xdim2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,16 +462,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.55637903260983</v>
+        <v>1.792445342185811e-05</v>
       </c>
       <c r="C2" t="n">
         <v>0.5450817913145818</v>
       </c>
       <c r="D2" t="n">
-        <v>0.01129724129524823</v>
+        <v>0.5450638668611599</v>
       </c>
       <c r="E2" t="n">
-        <v>2.07257726734964</v>
+        <v>99.99671160297272</v>
       </c>
     </row>
     <row r="3">
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6377961766522927</v>
+        <v>0.6295831446367834</v>
       </c>
       <c r="C3" t="n">
         <v>0.5938547655757322</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04394141107656047</v>
+        <v>0.0357283790610512</v>
       </c>
       <c r="E3" t="n">
-        <v>7.399353111860609</v>
+        <v>6.016349641719745</v>
       </c>
     </row>
     <row r="4">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.01824107477955189</v>
+        <v>0.5036173530585083</v>
       </c>
       <c r="C4" t="n">
         <v>0.0124333933545323</v>
       </c>
       <c r="D4" t="n">
-        <v>0.005807681425019593</v>
+        <v>0.491183959703976</v>
       </c>
       <c r="E4" t="n">
-        <v>46.7103489724512</v>
+        <v>3950.52215994539</v>
       </c>
     </row>
     <row r="5">
@@ -519,16 +519,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04999364893232866</v>
+        <v>0.1033797330328833</v>
       </c>
       <c r="C5" t="n">
         <v>0.05559015057568738</v>
       </c>
       <c r="D5" t="n">
-        <v>0.005596501643358717</v>
+        <v>0.0477895824571959</v>
       </c>
       <c r="E5" t="n">
-        <v>10.06743386265691</v>
+        <v>85.96771543572129</v>
       </c>
     </row>
     <row r="6">
@@ -538,16 +538,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.139638986097883</v>
+        <v>0.7609539008946413</v>
       </c>
       <c r="C6" t="n">
-        <v>0.07887393787074751</v>
+        <v>0.1119748681131919</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06076504822713549</v>
+        <v>0.6489790327814494</v>
       </c>
       <c r="E6" t="n">
-        <v>77.0407182239494</v>
+        <v>579.5756170263282</v>
       </c>
     </row>
     <row r="7">
@@ -557,111 +557,73 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.06206019134593488</v>
+        <v>0.3693657949527629</v>
       </c>
       <c r="C7" t="n">
-        <v>0.07644290486368606</v>
+        <v>0.1059701059804418</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01438271351775118</v>
+        <v>0.2633956889723211</v>
       </c>
       <c r="E7" t="n">
-        <v>18.81497510252732</v>
+        <v>248.556596726377</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>kappa_p1</t>
+          <t>lambda1</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0530931394238478</v>
+        <v>0.02531112445337835</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6450817913145818</v>
+        <v>0.352759752057376</v>
       </c>
       <c r="D8" t="n">
-        <v>0.591988651890734</v>
+        <v>0.3274486276039976</v>
       </c>
       <c r="E8" t="n">
-        <v>91.7695492046595</v>
+        <v>92.82482644186076</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>kappa_p2</t>
+          <t>lambda2</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8722777460490261</v>
+        <v>2.96012599854123e-06</v>
       </c>
       <c r="C9" t="n">
-        <v>0.6938547655757322</v>
+        <v>0.1597769708385401</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1784229804732939</v>
+        <v>0.1597740107125416</v>
       </c>
       <c r="E9" t="n">
-        <v>25.71474454387379</v>
+        <v>99.99814733876666</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>theta_p1</t>
+          <t>sigma_err</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.3509077016172114</v>
+        <v>0.01993599323705686</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0224333933545323</v>
+        <v>0.005798495327151224</v>
       </c>
       <c r="D10" t="n">
-        <v>0.328474308262679</v>
+        <v>0.01413749790990564</v>
       </c>
       <c r="E10" t="n">
-        <v>1464.220339168244</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>theta_p2</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.03572307294603616</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.06559015057568737</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.02986707762965121</v>
-      </c>
-      <c r="E11" t="n">
-        <v>45.53591868215987</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>sigma_err</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1.37380250836705e-05</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.004307391579211622</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.004293653554127952</v>
-      </c>
-      <c r="E12" t="n">
-        <v>99.6810592946791</v>
+        <v>243.8132155372681</v>
       </c>
     </row>
   </sheetData>

</xml_diff>